<commit_message>
updated daily rejection data
</commit_message>
<xml_diff>
--- a/rejection_data.xlsx
+++ b/rejection_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Admin\Desktop\PistonRodPortal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6CE5709-106C-4B2A-A94A-2D6E9B33672E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60D348E-FEBD-4F02-9CE4-36648D82312E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2FF8ABF7-B34E-4442-953A-A8AB69CBC555}"/>
   </bookViews>
@@ -708,7 +708,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -716,13 +716,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1217,18 +1210,6 @@
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>12.099227708869646</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>11.976187308766795</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>13.121998078770414</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>10.06338028169014</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>9.7628304821150849</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>0</c:v>
@@ -1700,18 +1681,6 @@
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0.5289024104844372</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.35253425568710922</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0.40666026256804355</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0.27464788732394368</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0.90590979782270609</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>0</c:v>
@@ -3872,14 +3841,14 @@
       </c>
       <c r="D5" s="21">
         <f>AM5/AM22*100</f>
-        <v>1.396017286126338</v>
+        <v>1.3597491089083971</v>
       </c>
       <c r="E5" s="22">
         <v>1.74</v>
       </c>
       <c r="F5" s="23">
         <f>SUM(H5:AL5)</f>
-        <v>6955</v>
+        <v>5398</v>
       </c>
       <c r="G5" s="24">
         <v>15722</v>
@@ -3947,22 +3916,10 @@
         <f>116+80+84+87</f>
         <v>367</v>
       </c>
-      <c r="Y5" s="25">
-        <f>56+87+40+188</f>
-        <v>371</v>
-      </c>
-      <c r="Z5" s="25">
-        <f>251+177+83+134</f>
-        <v>645</v>
-      </c>
-      <c r="AA5" s="25">
-        <f>122+54</f>
-        <v>176</v>
-      </c>
-      <c r="AB5" s="25">
-        <f>96+65+74+130</f>
-        <v>365</v>
-      </c>
+      <c r="Y5" s="25"/>
+      <c r="Z5" s="25"/>
+      <c r="AA5" s="25"/>
+      <c r="AB5" s="25"/>
       <c r="AC5" s="26"/>
       <c r="AD5" s="26"/>
       <c r="AE5" s="25"/>
@@ -3975,7 +3932,7 @@
       <c r="AL5" s="25"/>
       <c r="AM5" s="25">
         <f>SUM(H5:AL5)</f>
-        <v>6955</v>
+        <v>5398</v>
       </c>
     </row>
     <row r="6" spans="2:175" s="31" customFormat="1" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4049,18 +4006,10 @@
       <c r="X6" s="29">
         <v>0</v>
       </c>
-      <c r="Y6" s="29">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="29">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="29">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="29">
-        <v>0</v>
-      </c>
+      <c r="Y6" s="29"/>
+      <c r="Z6" s="29"/>
+      <c r="AA6" s="29"/>
+      <c r="AB6" s="29"/>
       <c r="AC6" s="29"/>
       <c r="AD6" s="29"/>
       <c r="AE6" s="29"/>
@@ -4220,7 +4169,7 @@
       </c>
       <c r="D7" s="21">
         <f>AM7/AM24*100</f>
-        <v>133.32075597926075</v>
+        <v>134.21574220813523</v>
       </c>
       <c r="E7" s="22">
         <v>0.33</v>
@@ -4281,18 +4230,10 @@
       <c r="X7" s="33">
         <v>0</v>
       </c>
-      <c r="Y7" s="33">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="33">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="33">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="33">
-        <v>0</v>
-      </c>
+      <c r="Y7" s="33"/>
+      <c r="Z7" s="33"/>
+      <c r="AA7" s="33"/>
+      <c r="AB7" s="33"/>
       <c r="AC7" s="34"/>
       <c r="AD7" s="34"/>
       <c r="AE7" s="33"/>
@@ -4318,14 +4259,14 @@
       </c>
       <c r="D8" s="21">
         <f>AM8/AM22*100</f>
-        <v>1.7366414895133107</v>
+        <v>1.7527110596118241</v>
       </c>
       <c r="E8" s="22">
         <v>0.51</v>
       </c>
       <c r="F8" s="23">
         <f t="shared" si="1"/>
-        <v>8652</v>
+        <v>6958</v>
       </c>
       <c r="G8" s="24">
         <v>4592</v>
@@ -4393,22 +4334,10 @@
         <f>250+44+98</f>
         <v>392</v>
       </c>
-      <c r="Y8" s="30">
-        <f>210+111+377</f>
-        <v>698</v>
-      </c>
-      <c r="Z8" s="30">
-        <f>115+129+90+211</f>
-        <v>545</v>
-      </c>
-      <c r="AA8" s="36">
-        <f>136+0</f>
-        <v>136</v>
-      </c>
-      <c r="AB8" s="30">
-        <f>158+87+70</f>
-        <v>315</v>
-      </c>
+      <c r="Y8" s="30"/>
+      <c r="Z8" s="30"/>
+      <c r="AA8" s="36"/>
+      <c r="AB8" s="30"/>
       <c r="AC8" s="38"/>
       <c r="AD8" s="38"/>
       <c r="AE8" s="30"/>
@@ -4421,7 +4350,7 @@
       <c r="AL8" s="30"/>
       <c r="AM8" s="30">
         <f t="shared" si="2"/>
-        <v>8652</v>
+        <v>6958</v>
       </c>
     </row>
     <row r="9" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4434,14 +4363,14 @@
       </c>
       <c r="D9" s="21">
         <f>AM9/AM22*100</f>
-        <v>0.29606405421083376</v>
+        <v>0.30253032230436921</v>
       </c>
       <c r="E9" s="22">
         <v>0.35</v>
       </c>
       <c r="F9" s="23">
         <f t="shared" si="1"/>
-        <v>1475</v>
+        <v>1201</v>
       </c>
       <c r="G9" s="24">
         <v>5267</v>
@@ -4509,22 +4438,10 @@
         <f>16+19+24</f>
         <v>59</v>
       </c>
-      <c r="Y9" s="30">
-        <f>14+40+39</f>
-        <v>93</v>
-      </c>
-      <c r="Z9" s="30">
-        <f>20+3+50+13</f>
-        <v>86</v>
-      </c>
-      <c r="AA9" s="30">
-        <f>12+15</f>
-        <v>27</v>
-      </c>
-      <c r="AB9" s="30">
-        <f>2+7+59</f>
-        <v>68</v>
-      </c>
+      <c r="Y9" s="30"/>
+      <c r="Z9" s="30"/>
+      <c r="AA9" s="30"/>
+      <c r="AB9" s="30"/>
       <c r="AC9" s="38"/>
       <c r="AD9" s="38"/>
       <c r="AE9" s="30"/>
@@ -4537,7 +4454,7 @@
       <c r="AL9" s="30"/>
       <c r="AM9" s="30">
         <f t="shared" si="2"/>
-        <v>1475</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="10" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4550,14 +4467,14 @@
       </c>
       <c r="D10" s="21">
         <f>AM10/AM22*100</f>
-        <v>0.18105069620215053</v>
+        <v>0.14685693414108844</v>
       </c>
       <c r="E10" s="22">
         <v>0.88</v>
       </c>
       <c r="F10" s="23">
         <f t="shared" si="1"/>
-        <v>902</v>
+        <v>583</v>
       </c>
       <c r="G10" s="24">
         <v>7891</v>
@@ -4615,20 +4532,10 @@
       <c r="X10" s="30">
         <v>10</v>
       </c>
-      <c r="Y10" s="30">
-        <f>27+8</f>
-        <v>35</v>
-      </c>
-      <c r="Z10" s="30">
-        <f>16+138+31</f>
-        <v>185</v>
-      </c>
-      <c r="AA10" s="30">
-        <v>5</v>
-      </c>
-      <c r="AB10" s="30">
-        <v>94</v>
-      </c>
+      <c r="Y10" s="30"/>
+      <c r="Z10" s="30"/>
+      <c r="AA10" s="30"/>
+      <c r="AB10" s="30"/>
       <c r="AC10" s="38"/>
       <c r="AD10" s="38"/>
       <c r="AE10" s="30"/>
@@ -4641,7 +4548,7 @@
       <c r="AL10" s="30"/>
       <c r="AM10" s="30">
         <f t="shared" si="2"/>
-        <v>902</v>
+        <v>583</v>
       </c>
     </row>
     <row r="11" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4654,14 +4561,14 @@
       </c>
       <c r="D11" s="21">
         <f>AM11/AM22*100</f>
-        <v>5.8729072285795141</v>
+        <v>5.8536216733629738</v>
       </c>
       <c r="E11" s="22">
         <v>0.59</v>
       </c>
       <c r="F11" s="23">
         <f t="shared" si="1"/>
-        <v>29259</v>
+        <v>23238</v>
       </c>
       <c r="G11" s="39">
         <v>5291</v>
@@ -4729,22 +4636,10 @@
         <f>742+69+205+131</f>
         <v>1147</v>
       </c>
-      <c r="Y11" s="30">
-        <f>232+355+700+231</f>
-        <v>1518</v>
-      </c>
-      <c r="Z11" s="30">
-        <f>180+550+650+858</f>
-        <v>2238</v>
-      </c>
-      <c r="AA11" s="30">
-        <f>500+486</f>
-        <v>986</v>
-      </c>
-      <c r="AB11" s="30">
-        <f>300+350+139+490</f>
-        <v>1279</v>
-      </c>
+      <c r="Y11" s="30"/>
+      <c r="Z11" s="30"/>
+      <c r="AA11" s="30"/>
+      <c r="AB11" s="30"/>
       <c r="AC11" s="38"/>
       <c r="AD11" s="38"/>
       <c r="AE11" s="30"/>
@@ -4757,7 +4652,7 @@
       <c r="AL11" s="30"/>
       <c r="AM11" s="30">
         <f t="shared" si="2"/>
-        <v>29259</v>
+        <v>23238</v>
       </c>
     </row>
     <row r="12" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4770,14 +4665,14 @@
       </c>
       <c r="D12" s="21">
         <f>AM12/AM22*100</f>
-        <v>0.86852146614934067</v>
+        <v>0.88189730090557572</v>
       </c>
       <c r="E12" s="22">
         <v>0.57999999999999996</v>
       </c>
       <c r="F12" s="23">
         <f t="shared" si="1"/>
-        <v>4327</v>
+        <v>3501</v>
       </c>
       <c r="G12" s="39">
         <v>5214</v>
@@ -4841,20 +4736,10 @@
         <f>100+41</f>
         <v>141</v>
       </c>
-      <c r="Y12" s="30">
-        <f>137+89+100</f>
-        <v>326</v>
-      </c>
-      <c r="Z12" s="30">
-        <f>100+200</f>
-        <v>300</v>
-      </c>
-      <c r="AA12" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="30">
-        <v>200</v>
-      </c>
+      <c r="Y12" s="30"/>
+      <c r="Z12" s="30"/>
+      <c r="AA12" s="30"/>
+      <c r="AB12" s="30"/>
       <c r="AC12" s="38"/>
       <c r="AD12" s="38"/>
       <c r="AE12" s="30"/>
@@ -4867,7 +4752,7 @@
       <c r="AL12" s="41"/>
       <c r="AM12" s="41">
         <f t="shared" si="2"/>
-        <v>4327</v>
+        <v>3501</v>
       </c>
     </row>
     <row r="13" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4880,14 +4765,14 @@
       </c>
       <c r="D13" s="21">
         <f>AM13/AM22*100</f>
-        <v>1.2727743510175571</v>
+        <v>1.2242276156529845</v>
       </c>
       <c r="E13" s="22">
         <v>0.36</v>
       </c>
       <c r="F13" s="23">
         <f t="shared" si="1"/>
-        <v>6341</v>
+        <v>4860</v>
       </c>
       <c r="G13" s="39">
         <v>3248</v>
@@ -4955,22 +4840,10 @@
         <f>0+286+201+39+30</f>
         <v>556</v>
       </c>
-      <c r="Y13" s="30">
-        <f>464+149+56+60</f>
-        <v>729</v>
-      </c>
-      <c r="Z13" s="30">
-        <f>249+63+40</f>
-        <v>352</v>
-      </c>
-      <c r="AA13" s="30">
-        <f>26+40</f>
-        <v>66</v>
-      </c>
-      <c r="AB13" s="30">
-        <f>30+25+40+239</f>
-        <v>334</v>
-      </c>
+      <c r="Y13" s="30"/>
+      <c r="Z13" s="30"/>
+      <c r="AA13" s="30"/>
+      <c r="AB13" s="30"/>
       <c r="AC13" s="38"/>
       <c r="AD13" s="38"/>
       <c r="AE13" s="30"/>
@@ -4983,7 +4856,7 @@
       <c r="AL13" s="30"/>
       <c r="AM13" s="30">
         <f t="shared" si="2"/>
-        <v>6341</v>
+        <v>4860</v>
       </c>
     </row>
     <row r="14" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4998,7 +4871,7 @@
       <c r="E14" s="22"/>
       <c r="F14" s="23">
         <f t="shared" si="1"/>
-        <v>704</v>
+        <v>352</v>
       </c>
       <c r="G14" s="39"/>
       <c r="H14" s="30"/>
@@ -5051,19 +4924,10 @@
       <c r="X14" s="30">
         <v>0</v>
       </c>
-      <c r="Y14" s="30">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="30">
-        <f>40+63+249</f>
-        <v>352</v>
-      </c>
-      <c r="AA14" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="30">
-        <v>0</v>
-      </c>
+      <c r="Y14" s="30"/>
+      <c r="Z14" s="30"/>
+      <c r="AA14" s="30"/>
+      <c r="AB14" s="30"/>
       <c r="AC14" s="38"/>
       <c r="AD14" s="38"/>
       <c r="AE14" s="30"/>
@@ -5076,7 +4940,7 @@
       <c r="AL14" s="30"/>
       <c r="AM14" s="30">
         <f t="shared" si="2"/>
-        <v>704</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5089,14 +4953,14 @@
       </c>
       <c r="D15" s="21">
         <f>AM15/AM22*100</f>
-        <v>0.37394395457273444</v>
+        <v>0.39548093756691061</v>
       </c>
       <c r="E15" s="22">
         <v>0.17</v>
       </c>
       <c r="F15" s="23">
         <f t="shared" si="1"/>
-        <v>1863</v>
+        <v>1570</v>
       </c>
       <c r="G15" s="39">
         <v>1489</v>
@@ -5164,22 +5028,10 @@
         <f>5+23+26</f>
         <v>54</v>
       </c>
-      <c r="Y15" s="30">
-        <f>103+4+50</f>
-        <v>157</v>
-      </c>
-      <c r="Z15" s="30">
-        <f>20+27</f>
-        <v>47</v>
-      </c>
-      <c r="AA15" s="30">
-        <f>10+23</f>
-        <v>33</v>
-      </c>
-      <c r="AB15" s="30">
-        <f>16+20+20</f>
-        <v>56</v>
-      </c>
+      <c r="Y15" s="30"/>
+      <c r="Z15" s="30"/>
+      <c r="AA15" s="30"/>
+      <c r="AB15" s="30"/>
       <c r="AC15" s="38"/>
       <c r="AD15" s="38"/>
       <c r="AE15" s="30"/>
@@ -5192,7 +5044,7 @@
       <c r="AL15" s="30"/>
       <c r="AM15" s="30">
         <f t="shared" si="2"/>
-        <v>1863</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="16" spans="2:175" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5265,18 +5117,10 @@
       <c r="X16" s="37">
         <v>0</v>
       </c>
-      <c r="Y16" s="37">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="37">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="37">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="37">
-        <v>0</v>
-      </c>
+      <c r="Y16" s="37"/>
+      <c r="Z16" s="37"/>
+      <c r="AA16" s="37"/>
+      <c r="AB16" s="37"/>
       <c r="AC16" s="37"/>
       <c r="AD16" s="37"/>
       <c r="AE16" s="37"/>
@@ -5302,7 +5146,7 @@
       </c>
       <c r="D17" s="21">
         <f>AM17/AM22*100</f>
-        <v>7.0252487439858855E-3</v>
+        <v>8.8164540221922737E-3</v>
       </c>
       <c r="E17" s="22">
         <v>0.01</v>
@@ -5363,18 +5207,10 @@
       <c r="X17" s="37">
         <v>0</v>
       </c>
-      <c r="Y17" s="37">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="37">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="37">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="37">
-        <v>0</v>
-      </c>
+      <c r="Y17" s="37"/>
+      <c r="Z17" s="37"/>
+      <c r="AA17" s="37"/>
+      <c r="AB17" s="37"/>
       <c r="AC17" s="43"/>
       <c r="AD17" s="43"/>
       <c r="AE17" s="37"/>
@@ -5400,14 +5236,14 @@
       </c>
       <c r="D18" s="21">
         <f>AM18/AM22*100</f>
-        <v>0.22942455183931049</v>
+        <v>0.24308223232615842</v>
       </c>
       <c r="E18" s="22">
         <v>0.21</v>
       </c>
       <c r="F18" s="23">
         <f t="shared" si="1"/>
-        <v>1143</v>
+        <v>965</v>
       </c>
       <c r="G18" s="39">
         <v>1872</v>
@@ -5475,22 +5311,10 @@
         <f>6+26+26</f>
         <v>58</v>
       </c>
-      <c r="Y18" s="37">
-        <f>48+22</f>
-        <v>70</v>
-      </c>
-      <c r="Z18" s="37">
-        <f>16+20</f>
-        <v>36</v>
-      </c>
-      <c r="AA18" s="37">
-        <f>28+11</f>
-        <v>39</v>
-      </c>
-      <c r="AB18" s="37">
-        <f>20+13</f>
-        <v>33</v>
-      </c>
+      <c r="Y18" s="37"/>
+      <c r="Z18" s="37"/>
+      <c r="AA18" s="37"/>
+      <c r="AB18" s="37"/>
       <c r="AC18" s="43"/>
       <c r="AD18" s="43"/>
       <c r="AE18" s="37"/>
@@ -5503,7 +5327,7 @@
       <c r="AL18" s="37"/>
       <c r="AM18" s="37">
         <f t="shared" si="2"/>
-        <v>1143</v>
+        <v>965</v>
       </c>
     </row>
     <row r="19" spans="1:41" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5516,14 +5340,14 @@
       </c>
       <c r="D19" s="21">
         <f>AM19/AM22*100</f>
-        <v>0.45403179025417351</v>
+        <v>0.48742395808405853</v>
       </c>
       <c r="E19" s="22">
         <v>0.28000000000000003</v>
       </c>
       <c r="F19" s="23">
         <f t="shared" si="1"/>
-        <v>2262</v>
+        <v>1935</v>
       </c>
       <c r="G19" s="39">
         <v>2502</v>
@@ -5585,20 +5409,10 @@
       <c r="X19" s="44">
         <v>55</v>
       </c>
-      <c r="Y19" s="44">
-        <f>35+1</f>
-        <v>36</v>
-      </c>
-      <c r="Z19" s="44">
-        <f>41+50</f>
-        <v>91</v>
-      </c>
-      <c r="AA19" s="37">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="37">
-        <v>200</v>
-      </c>
+      <c r="Y19" s="44"/>
+      <c r="Z19" s="44"/>
+      <c r="AA19" s="37"/>
+      <c r="AB19" s="37"/>
       <c r="AC19" s="43"/>
       <c r="AD19" s="43"/>
       <c r="AE19" s="37"/>
@@ -5611,7 +5425,7 @@
       <c r="AL19" s="37"/>
       <c r="AM19" s="37">
         <f t="shared" si="2"/>
-        <v>2262</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="20" spans="1:41" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5684,18 +5498,10 @@
       <c r="X20" s="44">
         <v>0</v>
       </c>
-      <c r="Y20" s="44">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="44">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="44">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="44">
-        <v>0</v>
-      </c>
+      <c r="Y20" s="44"/>
+      <c r="Z20" s="44"/>
+      <c r="AA20" s="44"/>
+      <c r="AB20" s="44"/>
       <c r="AC20" s="44"/>
       <c r="AD20" s="44"/>
       <c r="AE20" s="44"/>
@@ -5781,18 +5587,10 @@
       <c r="X21" s="44">
         <v>0</v>
       </c>
-      <c r="Y21" s="44">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="44">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="44">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="44">
-        <v>0</v>
-      </c>
+      <c r="Y21" s="44"/>
+      <c r="Z21" s="44"/>
+      <c r="AA21" s="44"/>
+      <c r="AB21" s="44"/>
       <c r="AC21" s="44"/>
       <c r="AD21" s="44"/>
       <c r="AE21" s="44"/>
@@ -5815,14 +5613,14 @@
       <c r="C22" s="46"/>
       <c r="D22" s="47">
         <f>D5+D6+D7+D8+D9+D10+D11+D12+D13+D15+D16+D17+D18+D19+D20+D21</f>
-        <v>146.00915809647</v>
+        <v>146.8721398050217</v>
       </c>
       <c r="E22" s="22">
         <v>0.5</v>
       </c>
       <c r="F22" s="23">
         <f t="shared" si="1"/>
-        <v>498203</v>
+        <v>396985</v>
       </c>
       <c r="G22" s="46"/>
       <c r="H22" s="29"/>
@@ -5888,22 +5686,10 @@
         <f>6071+3300+6450+5544</f>
         <v>21365</v>
       </c>
-      <c r="Y22" s="29">
-        <f>6900+6420+6280+10468</f>
-        <v>30068</v>
-      </c>
-      <c r="Z22" s="29">
-        <f>5840+6780+10200+8410</f>
-        <v>31230</v>
-      </c>
-      <c r="AA22" s="48">
-        <f>7000+7200</f>
-        <v>14200</v>
-      </c>
-      <c r="AB22" s="48">
-        <f>5600+7200+4620+8300</f>
-        <v>25720</v>
-      </c>
+      <c r="Y22" s="29"/>
+      <c r="Z22" s="29"/>
+      <c r="AA22" s="48"/>
+      <c r="AB22" s="48"/>
       <c r="AC22" s="49"/>
       <c r="AD22" s="49"/>
       <c r="AE22" s="48"/>
@@ -5916,7 +5702,7 @@
       <c r="AL22" s="29"/>
       <c r="AM22" s="30">
         <f>SUM(H22:AL22)</f>
-        <v>498203</v>
+        <v>396985</v>
       </c>
     </row>
     <row r="23" spans="1:41" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5997,22 +5783,10 @@
         <f t="shared" si="4"/>
         <v>2585</v>
       </c>
-      <c r="Y23" s="52">
-        <f t="shared" si="4"/>
-        <v>3601</v>
-      </c>
-      <c r="Z23" s="52">
-        <f t="shared" si="4"/>
-        <v>4098</v>
-      </c>
-      <c r="AA23" s="52">
-        <f t="shared" si="4"/>
-        <v>1429</v>
-      </c>
-      <c r="AB23" s="52">
-        <f t="shared" si="4"/>
-        <v>2511</v>
-      </c>
+      <c r="Y23" s="52"/>
+      <c r="Z23" s="52"/>
+      <c r="AA23" s="52"/>
+      <c r="AB23" s="52"/>
       <c r="AC23" s="52">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -6055,7 +5829,7 @@
       </c>
       <c r="AM23" s="53">
         <f>(+AM15+AM13+AM11+AM12+AM10+AM9+AM8+AM5+AM7+AM6)</f>
-        <v>59790</v>
+        <v>47325</v>
       </c>
       <c r="AN23" s="54"/>
       <c r="AO23" s="55"/>
@@ -6142,22 +5916,10 @@
         <f t="shared" si="6"/>
         <v>12.099227708869646</v>
       </c>
-      <c r="Y24" s="57">
-        <f t="shared" si="6"/>
-        <v>11.976187308766795</v>
-      </c>
-      <c r="Z24" s="57">
-        <f t="shared" si="6"/>
-        <v>13.121998078770414</v>
-      </c>
-      <c r="AA24" s="57">
-        <f t="shared" si="6"/>
-        <v>10.06338028169014</v>
-      </c>
-      <c r="AB24" s="57">
-        <f t="shared" si="6"/>
-        <v>9.7628304821150849</v>
-      </c>
+      <c r="Y24" s="57"/>
+      <c r="Z24" s="57"/>
+      <c r="AA24" s="57"/>
+      <c r="AB24" s="57"/>
       <c r="AC24" s="57" t="e">
         <f t="shared" si="6"/>
         <v>#DIV/0!</v>
@@ -6197,7 +5959,7 @@
       </c>
       <c r="AM24" s="58">
         <f>+AM23/AM22*100</f>
-        <v>12.001132068654744</v>
+        <v>11.921105331435697</v>
       </c>
       <c r="AN24" s="59"/>
       <c r="AO24" s="55"/>
@@ -6280,22 +6042,10 @@
         <f t="shared" si="7"/>
         <v>113</v>
       </c>
-      <c r="Y25" s="61">
-        <f t="shared" si="7"/>
-        <v>106</v>
-      </c>
-      <c r="Z25" s="61">
-        <f t="shared" si="7"/>
-        <v>127</v>
-      </c>
-      <c r="AA25" s="61">
-        <f t="shared" si="7"/>
-        <v>39</v>
-      </c>
-      <c r="AB25" s="61">
-        <f t="shared" si="7"/>
-        <v>233</v>
-      </c>
+      <c r="Y25" s="61"/>
+      <c r="Z25" s="61"/>
+      <c r="AA25" s="61"/>
+      <c r="AB25" s="61"/>
       <c r="AC25" s="61">
         <f t="shared" si="7"/>
         <v>0</v>
@@ -6335,7 +6085,7 @@
       </c>
       <c r="AM25" s="30">
         <f>SUM(H25:AL25)</f>
-        <v>3440</v>
+        <v>2935</v>
       </c>
       <c r="AN25" s="59"/>
       <c r="AO25" s="55"/>
@@ -6422,22 +6172,10 @@
         <f t="shared" si="8"/>
         <v>0.5289024104844372</v>
       </c>
-      <c r="Y26" s="63">
-        <f t="shared" si="8"/>
-        <v>0.35253425568710922</v>
-      </c>
-      <c r="Z26" s="63">
-        <f t="shared" si="8"/>
-        <v>0.40666026256804355</v>
-      </c>
-      <c r="AA26" s="63">
-        <f t="shared" si="8"/>
-        <v>0.27464788732394368</v>
-      </c>
-      <c r="AB26" s="63">
-        <f t="shared" si="8"/>
-        <v>0.90590979782270609</v>
-      </c>
+      <c r="Y26" s="63"/>
+      <c r="Z26" s="63"/>
+      <c r="AA26" s="63"/>
+      <c r="AB26" s="63"/>
       <c r="AC26" s="63" t="e">
         <f t="shared" si="8"/>
         <v>#DIV/0!</v>
@@ -6477,7 +6215,7 @@
       </c>
       <c r="AM26" s="58">
         <f>(AM25/AM22*100)</f>
-        <v>0.69048159083746985</v>
+        <v>0.73932264443240936</v>
       </c>
       <c r="AN26" s="64"/>
       <c r="AO26" s="55"/>

</xml_diff>